<commit_message>
Add eight source-reviewed Renmin University profiles (790 total)
</commit_message>
<xml_diff>
--- a/site/exports/ruc-sociology.xlsx
+++ b/site/exports/ruc-sociology.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -675,12 +675,120 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>社会学院</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>仅保留必要职业摘录，非完整网页或原始HTTP档案；观察窗口或完成端点不是独立认证的精确请求时刻。；独立师资目录、当前人事与退休状态未核；现任和开放任期仅来源标签，导航关闭。；本人导师、原学位证书与论文未核，不由教授等职业称谓推本人师承。；选录成果不代表全部作品；未核出版者元数据、完整作者/编辑名单或知识产权登记。；官网标签教授；2018.08起社会与人口学院社会学系教授为原历史任职句，与当前页面标题“社会学院”分别保留，不推更名、重组或实时任职。；博士生2001—2004、硕士生1998—2001及本科生1994—1998均为学生阶段，无独立授位陈述；社会学系保留在机构名中，专业未知。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>赵延东</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>社会学院</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>仅保留必要职业摘录，非完整网页或原始HTTP档案；观察窗口或完成端点不是独立认证的精确请求时刻。；独立师资目录、当前人事与退休状态未核；现任和开放任期仅来源标签，导航关闭。；本人导师、原学位证书与论文未核，不由教授等职业称谓推本人师承。；选录成果不代表全部作品；未核出版者元数据、完整作者/编辑名单或知识产权登记。；官网社会学院页面标题、具名赵延东及教授标签支持展示归属，未留存明确本人任职句，不产生雇佣或任职事件。原标题/姓名/职称为分列字段拼接，非连续原句。；中国社会科学院研究生院、华中科技大学、中南财经政法大学及原系名照录，不独立修正历史校名；博士、硕士、学士明确获授但日期未知。</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -692,11 +800,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="29.4" customWidth="1" min="2" max="2"/>
+    <col width="40.59999999999999" customWidth="1" min="2" max="2"/>
     <col width="19.6" customWidth="1" min="3" max="3"/>
     <col width="23.8" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -2277,8 +2385,540 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>education_label_award_unknown</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>博士生</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>北京大学社会学系</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>官网为学生阶段标签，保留教育经历但授位状态未知；机构中的系名不独立认证所学专业。</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>education_label_award_unknown</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>硕士生</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>北京大学社会学系</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>官网为学生阶段标签，保留教育经历但授位状态未知；机构中的系名不独立认证所学专业。</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>education_label_award_unknown</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>本科生</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>吉林大学哲学社会学院社会学系</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>官网为学生阶段标签，保留教育经历但授位状态未知；机构中的系名不独立认证所学专业。</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_training</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>访问学者</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>美国乔治城大学</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>2012—2013美国乔治城大学访问学者，非学位经历；导师未知。</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2018-08</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>原职业标签和时段照录，当前任职未核，不补任期。</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr"/>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>赵延东</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>社会学博士</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>中国社会科学院研究生院社会学系</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>应用社会学</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>官网明确获学位，学习区间终点不当作授位日期，原证书未核。</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr"/>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>赵延东</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>法学硕士</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>华中科技大学社会学系</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>应用社会学</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>官网明确获学位，学习区间终点不当作授位日期，原证书未核。</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>赵延东</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>哲学学士</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>中南财经政法大学政法系</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>行政管理</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>官网明确获学位，学习区间终点不当作授位日期，原证书未核。</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="S33" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S25"/>
+  <autoFilter ref="A1:S33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -2304,6 +2944,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2406,19 +3054,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="18.2" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="57.4" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
@@ -2485,8 +3133,246 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>经济社会学研究（第三辑）</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>著作（执行主编）；book</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目，未外核。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>官网记2016年，社会科学文献出版社；本人贡献为执行主编，不等完整作者/编辑名单，不把主编或执行主编当作者。</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>王水雄</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>爱的策略——那代大学生的家庭关系与情感教育</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>著作（合著）；book</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目，未外核。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>官网记2016年，中华工商联合出版社；本人贡献为合著，不等完整作者/编辑名单，不把主编或执行主编当作者。</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>赵延东</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Science and Technology Governance and Ethics: A Global Perspective from Europe, India and China</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>著作（主编）；book</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目，未外核。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>官网记2014年，Springer；本人贡献为主编，不等完整作者/编辑名单，不把主编或执行主编当作者。</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>赵延东</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>第二次全国科技工作者状况调查报告</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>著作（合著）；book</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目，未外核。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>官网记2010年，中国科学技术出版社；本人贡献为合著，不等完整作者/编辑名单，不把主编或执行主编当作者。</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:L5"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId12"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2497,7 +3383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2771,27 +3657,23 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>陈那波</t>
+          <t>王水雄</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>institution-classification-2</t>
+          <t>ruc-wangshuixiong</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
-        </is>
-      </c>
+          <t>https://ssr.ruc.edu.cn/jszy/wsx/wsx_grjj/ae8aadab3aed46e5b6c2f51e37354b51.htm</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>未单独记录</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2808,42 +3690,112 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>赵延东</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ruc-zhaoyandong</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://ssr.ruc.edu.cn/jszy/zyd/zyd_grjj/b2d932587a0e4dc58796a0c8e2f67c85.htm</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>陈那波</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>institution-classification-2</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>未单独记录</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>中国人民大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>房莉杰</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>institution-classification-2</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>https://www.csust.edu.cn/fzgh/info/1016/1662.htm</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>未单独记录</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>ruc</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>ruc</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>中国人民大学</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -2853,6 +3805,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>